<commit_message>
Fix site-wide click bug in edition switch; edition selector moved into the profile menu (MVP default); new on-site Prompt interface; auto-detect Shard Cel art in art/shard/; world shows only MVP characters
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MVP Roster'!$A$1:$AG$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Prompts'!$A$1:$K$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Production Tracker'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Production Tracker'!$A$1:$L$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Slots'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Vote Scores'!$A$1:$F$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Changes'!$A$1:$B$10</definedName>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fill in as art is made. Dropdowns for status. The first sheet to open when you are drawing.</t>
+          <t>Fill in as art is made. Dropdowns for status, plus the exact file name to save each image as (art/shard/). The site finds the files on its own.</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6843,6 +6843,8 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6894,6 +6896,16 @@
       <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Original-style art exists?</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Save portrait as</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Save background as</t>
         </is>
       </c>
     </row>
@@ -6930,6 +6942,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/fuelpriests.png</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/fuelpriests-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -6964,6 +6986,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/pinball.png</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/pinball-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -6998,6 +7030,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/pipedpipers.png</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/pipedpipers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -7032,6 +7074,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/gargoyle.png</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/gargoyle-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -7066,6 +7118,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/batcallers.png</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/batcallers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -7100,6 +7162,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/bonecrushers.png</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/bonecrushers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -7134,6 +7206,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/flyingsquirrels.png</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/flyingsquirrels-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -7168,6 +7250,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/scarabshifters.png</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/scarabshifters-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -7202,6 +7294,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/rustwraith.png</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/rustwraith-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -7236,6 +7338,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/staticwraiths.png</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/staticwraiths-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -7270,6 +7382,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/seanceoperators.png</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/seanceoperators-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -7304,6 +7426,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/contractreapers.png</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/contractreapers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -7338,6 +7470,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/embalmeralchemists.png</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/embalmeralchemists-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -7372,6 +7514,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/marrowpuppeteers.png</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/marrowpuppeteers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -7406,6 +7558,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/canopybeastmasters.png</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/canopybeastmasters-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -7440,6 +7602,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/mossplate.png</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/mossplate-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -7474,6 +7646,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/nightmareshepherds.png</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/nightmareshepherds-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -7508,6 +7690,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/manymaw.png</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/manymaw-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -7542,6 +7734,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/etherwing.png</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/etherwing-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -7576,6 +7778,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/necromancers.png</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/necromancers-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -7610,6 +7822,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/stickywizards.png</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/stickywizards-bg.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -7644,9 +7866,19 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/sporecoven.png</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>art/shard/sporecoven-bg.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J23"/>
+  <autoFilter ref="A1:L23"/>
   <conditionalFormatting sqref="D2:D23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Approved"</formula>

</xml_diff>

<commit_message>
Neon Pied Pipers: new Shard Cel portrait and background; art text matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -1811,7 +1811,7 @@
       </c>
       <c r="Q4" s="6" t="inlineStr">
         <is>
-          <t>lanky showman in a pink neon jacket with huge shoulder pads over a cyan shirt, teal parachute pants and high-top boots, a synth-flute that is half flute and half keytar strapped across his chest, sunglasses pushed up in a teased hairdo, three small street-crew figures (a thief, a brawler, a lookout) dancing out of the music</t>
+          <t>lanky showman in a pink neon big-collar coat over a cyan shirt, teal baggy pants and huge pink-and-cream high-tops, goggles on a tall spiky black pompadour, a black-and-cyan keytar-flute with a piano keyboard on a strap, three small hooded crew members circled by glowing music notes</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>3681</v>
+        <v>3639</v>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
@@ -5289,7 +5289,7 @@
 IDENTITY: a lanky man in his thirties of Mexican heritage with a tall teased hairdo and sunglasses pushed up on his forehead.
 BODY: lanky and loose-limbed, huge shoulder pads, a tall teased hairdo build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. agile mover.
 FACE: cool, cocky half-smile.
-COSTUME: lanky showman in a pink neon jacket with huge shoulder pads over a cyan shirt, teal parachute pants and high-top boots, a synth-flute that is half flute and half keytar strapped across his chest, sunglasses pushed up in a teased hairdo, three small street-crew figures (a thief, a brawler, a lookout) dancing out of the music. Signature exaggeration: huge shoulder pads, giant high-top boots and an oversized synth-flute thrust forward.
+COSTUME: lanky showman in a pink neon big-collar coat over a cyan shirt, teal baggy pants and huge pink-and-cream high-tops, goggles on a tall spiky black pompadour, a black-and-cyan keytar-flute with a piano keyboard on a strap, three small hooded crew members circled by glowing music notes. Signature exaggeration: huge shoulder pads, giant high-top boots and an oversized synth-flute thrust forward.
 POSE: striding forward mid-riff with the synth-flute held out as three small crew members dance out of the music. Pose energy: arms flung wide or one hand commanding, small summoned allies bursting out around the figure drawn small and clearly separate, a strong S-curve body. Head turned toward the viewer. The pose must say "summoner" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -5311,7 +5311,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a barricaded highway-overpass settlement: stacked shipping containers, riveted gates, a tall radio mast, sodium street lamps, rain-slick asphalt, tarp banners.
-Scene props for Neon Pied Pipers: a neon-lit abandoned mall arcade with a pile of boomboxes, a roller-rink floor, graffiti walls, a small stage and strings of lights. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Neon Pied Pipers: a neon-lit overpass ruin under a yellow moon with stacked speaker cabinets, a row of arcade cabinets, a roller-rink floor with painted rings, a pink arched stage hall, a disco ball, teal banners, flight cases and strings of lights. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a GOLD-WASHED scene. The people color #d9a521 washes the whole scene (warm GOLD and amber: golden sky, gold-lit fog, gold light pooling on wet ground, gold-toned haze over everything), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #ff2e93 for the largest sign, banner or lit window band, SECONDARY #2de2e6 for several medium panels, flags or lights, POP #1b1035 for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Gargoyle Sentries: new Shard Cel portrait and background; art text matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -1974,7 +1974,7 @@
       </c>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>hunched vampire sentinel in a helmeted hood and a heavy wing-cloak, half the body gray carved stone and half pale cracked skin with small bat-wing horns, huge stone-knuckled fists planted on the ground, ledge-anchors on the belt</t>
+          <t>hunched vampire sentinel crouched on one huge stone fist, a blue hood with pointed ears over a pale cracked face with red eyes, giant stone-slab wings edged in crimson folded behind, one shoulder bare pale cracked skin and the rest gray stone, red-banded navy cuffs on stone-knuckled fists, a chain and a red sash at the belt</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -5359,14 +5359,14 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>3529</v>
+        <v>3626</v>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Gargoyle Sentries: a tank (soaks damage and holds the line), combat character, Vampire › Night Watch.
 BODY: squat and wide with a hunched hump back, huge hands, short legs, stone-slab shoulders build. Proportion recipe: large and bulky: blocky torso, small head sunk between huge shoulders, fists and feet twice natural size. climbing mover.
 FACE: grim, heavy-browed.
-COSTUME: hunched vampire sentinel in a helmeted hood and a heavy wing-cloak, half the body gray carved stone and half pale cracked skin with small bat-wing horns, huge stone-knuckled fists planted on the ground, ledge-anchors on the belt. Signature exaggeration: boulder-sized stone fists planted toward the viewer and a hunched hump back, the stone cracking into pale skin down one side.
+COSTUME: hunched vampire sentinel crouched on one huge stone fist, a blue hood with pointed ears over a pale cracked face with red eyes, giant stone-slab wings edged in crimson folded behind, one shoulder bare pale cracked skin and the rest gray stone, red-banded navy cuffs on stone-knuckled fists, a chain and a red sash at the belt. Signature exaggeration: boulder-sized stone fists planted toward the viewer and a hunched hump back, the stone cracking into pale skin down one side.
 POSE: perched on all fours on a ledge edge, the wings folded like a cloak, the head thrust forward, the fists planted. Pose energy: a planted wide low stance, the shield or fist thrust toward the viewer and drawn huge, weight sunk into the legs, a chunky layered silhouette. Head turned toward the viewer. The pose must say "tank" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -5388,7 +5388,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a gutted skyscraper rooftop at night: a chandelier wired to car batteries, a dead neon sign, gothic antenna spires, a distant ruined skyline, rain.
-Scene props for Gargoyle Sentries: a gothic ledge of a skyscraper roof with stone gargoyle statues, a stone parapet, rain gutters, a clock tower, a crane arm. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Gargoyle Sentries: a rain-soaked gothic rooftop under a pale moon with stone gargoyle statues on plinths, a gothic balustrade, glowing red lantern posts, a hanging chandelier with blue flames, a clock tower, a crane arm, a gothic spire skyline and a glowing blue banner panel. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a BLACK-WASHED scene. The people color #16161c washes the whole scene (deep INK BLACK: near-black sky, ground and architecture in layered blacks and charcoal, only a few thin grey highlights), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. Because this people is near-black, keep the wash in layered flat blacks and charcoals with thin grey rim shapes. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #8bb9e5 for the largest sign, banner or lit window band, SECONDARY #ff4d6d for several medium panels, flags or lights, POP #023054 for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Belfry Batcallers: new Shard Cel portrait and background; art text matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -2141,7 +2141,7 @@
       </c>
       <c r="Q6" s="6" t="inlineStr">
         <is>
-          <t>tall gaunt vampire with a high collar, a long violet bat-wing cloak, a thin black bodice and boots, a small silver bell in one hand, five small bats peeling off the cloak around her</t>
+          <t>tall gaunt vampire with a tall white crown-swept hairdo and pointed ears, a huge violet bat-wing cloak lined in lavender and edged in crimson shards, a black plunging bodice and thigh-high spiked boots, a silver bell in one hand, the other hand raised, five small black bats with crimson wings circling her</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>3518</v>
+        <v>3643</v>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
@@ -5444,7 +5444,7 @@
 IDENTITY: a gaunt woman in her sixties of Hungarian heritage with a high white widow's peak.
 BODY: very tall and thin, a swan neck, a huge bat-wing cloak that doubles the width build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. flying mover.
 FACE: serene, almost smiling.
-COSTUME: tall gaunt vampire with a high collar, a long violet bat-wing cloak, a thin black bodice and boots, a small silver bell in one hand, five small bats peeling off the cloak around her. Signature exaggeration: a huge bat-wing cloak fanned wide into points and an oversized silver bell in one hand.
+COSTUME: tall gaunt vampire with a tall white crown-swept hairdo and pointed ears, a huge violet bat-wing cloak lined in lavender and edged in crimson shards, a black plunging bodice and thigh-high spiked boots, a silver bell in one hand, the other hand raised, five small black bats with crimson wings circling her. Signature exaggeration: a huge bat-wing cloak fanned wide into points and an oversized silver bell in one hand.
 POSE: arms flung wide on tiptoe as a swarm of bats peels away from the cloak, the bell held out in one hand. Pose energy: arms flung wide or one hand commanding, small summoned allies bursting out around the figure drawn small and clearly separate, a strong S-curve body. Head turned toward the viewer. The pose must say "summoner" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -5466,7 +5466,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a gutted skyscraper rooftop at night: a chandelier wired to car batteries, a dead neon sign, gothic antenna spires, a distant ruined skyline, rain.
-Scene props for Belfry Batcallers: a ruined bell-loft with a huge cracked bell, rope pulls, stone gargoyles, hanging bat roosts and a broken stained-glass window. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Belfry Batcallers: a rainy gothic bell-loft under a pale moon with a huge cracked bell on chains, tall violet stained-glass windows, stone gargoyle statues on plinths, red candle clusters and hanging cage lanterns, a gothic balustrade, torn violet banners and a spire skyline. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a BLACK-WASHED scene. The people color #16161c washes the whole scene (deep INK BLACK: near-black sky, ground and architecture in layered blacks and charcoal, only a few thin grey highlights), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. Because this people is near-black, keep the wash in layered flat blacks and charcoals with thin grey rim shapes. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #52358d for the largest sign, banner or lit window band, SECONDARY #d9d2f0 for several medium panels, flags or lights, POP #ff4b6e for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Scarab Shifters: new Shard Cel portrait and background; art text matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -2669,7 +2669,7 @@
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>tall lean were-beetle half-shifted, green-black carapace plates on the shoulders and forearms, golden wing-cases half open on the back, small mandibles at the jaw, a gold scarab pendant and wrapped belt, one cupped hand pouring a swarm of small scarabs</t>
+          <t>tall lean were-beetle half-shifted, a green beetle-horn crown headdress, a gold scarab pendant, huge green-black carapace shoulder plates, a giant gold-clawed gauntlet, golden wing-cases flared on the back, a white-and-green striped kilt and pants with gold trim, clawed beetle boots, a swarm of green-and-gold scarabs pouring from one hand</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -5668,7 +5668,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>3672</v>
+        <v>3760</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
@@ -5676,7 +5676,7 @@
 IDENTITY: a tall lean man in his late twenties of Egyptian heritage mid-shift, with beetle mandibles at the jaw.
 BODY: tall and lean, glossy carapace plates grown over the shoulders and forearms, wing-cases folded on the back build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. flying mover.
 FACE: intense, half-changed.
-COSTUME: tall lean were-beetle half-shifted, green-black carapace plates on the shoulders and forearms, golden wing-cases half open on the back, small mandibles at the jaw, a gold scarab pendant and wrapped belt, one cupped hand pouring a swarm of small scarabs. Signature exaggeration: an oversized beetle-plate gauntlet and shoulder, golden wing-cases flared, and a swarm bursting from the cupped hand.
+COSTUME: tall lean were-beetle half-shifted, a green beetle-horn crown headdress, a gold scarab pendant, huge green-black carapace shoulder plates, a giant gold-clawed gauntlet, golden wing-cases flared on the back, a white-and-green striped kilt and pants with gold trim, clawed beetle boots, a swarm of green-and-gold scarabs pouring from one hand. Signature exaggeration: an oversized beetle-plate gauntlet and shoulder, golden wing-cases flared, and a swarm bursting from the cupped hand.
 POSE: crouched mid-shift with one hand cupped as scarabs pour out and the other arm armored in beetle plates. Pose energy: arms flung wide or one hand commanding, small summoned allies bursting out around the figure drawn small and clearly separate, a strong S-curve body. Head turned toward the viewer. The pose must say "summoner" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -5698,7 +5698,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a scrapyard war-den of rusted buses and tire-wall palisades, campfire barrels, hand-painted war totems, signal horns on tall poles.
-Scene props for Scarab Shifters: a sunlit scrapyard dune with half-buried car bodies, a dung-ball mound, a rusted gate arch, tall dry grass and a dust haze. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Scarab Shifters: a sunlit scrapyard dune under a pale moon with a rusted gate arch with a sun sigil, a half-buried bus body, a spiked dome of scrap, giant curved bone tusks, loudspeaker horns on poles, green and gold banners and tall dry grass. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a RUST-WASHED scene. The people color #b4532a washes the whole scene (burnt RUST and copper orange: rust-tinted sky, orange-brown haze, copper light on the ground), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #0f7d5a for the largest sign, banner or lit window band, SECONDARY #e8b923 for several medium panels, flags or lights, POP #1a1a1a for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Marrow Puppeteers: new Shard Cel portrait and background; figure text matched
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -3619,7 +3619,7 @@
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>tall skeletal conductor in a magenta tailcoat with bone-white cuffs, a bone baton in one hand, glowing bone-white strings running from his fingers to a crow and a wolf at his feet, their ribs shining through</t>
+          <t>tall grinning skeletal conductor in a magenta top hat and tailcoat with bone-white cuffs and a chain at the belt, a bone baton raised in one hand, glowing bone-white strings running from his fingers to a crow and a wolf at his feet, their ribs shining through</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -6132,7 +6132,7 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>3568</v>
+        <v>3620</v>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
@@ -6140,7 +6140,7 @@
 IDENTITY: a long, skeletal man of ancient age in a conductor's tailcoat, once a street performer in Cairo.
 BODY: stretched and doll-jointed, arms too long, a tailcoat that ends in splinters build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. grounded mover.
 FACE: gleeful, hollow-eyed concentration.
-COSTUME: tall skeletal conductor in a magenta tailcoat with bone-white cuffs, a bone baton in one hand, glowing bone-white strings running from his fingers to a crow and a wolf at his feet, their ribs shining through. Signature exaggeration: overlong splayed fingers with glowing strings stretching toward the viewer and a splintered tailcoat.
+COSTUME: tall grinning skeletal conductor in a magenta top hat and tailcoat with bone-white cuffs and a chain at the belt, a bone baton raised in one hand, glowing bone-white strings running from his fingers to a crow and a wolf at his feet, their ribs shining through. Signature exaggeration: overlong splayed fingers with glowing strings stretching toward the viewer and a splintered tailcoat.
 POSE: hunched forward, both hands splayed with glowing strings running to a crow and a wolf. Pose energy: arms flung wide or one hand commanding, small summoned allies bursting out around the figure drawn small and clearly separate, a strong S-curve body. Head turned toward the viewer. The pose must say "summoner" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.

</xml_diff>

<commit_message>
Canopy Beastmasters: new Shard Cel portrait and background; art text matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -3782,7 +3782,7 @@
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>tall woman with an antler crown and braided hair in a green leaf-cloak and straps, a carved horn at her lips, a fox, an owl, a small panther and a monkey gathered at her feet and shoulders</t>
+          <t>tall woman with an antler crown and long black braids, a huge maroon-and-gold feather cloak with green leaf trim, a claw-tooth belt and striped boots, a big carved horn at her lips, an owl on her shoulder, a monkey on her back, a black panther and a fox at her feet</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -6210,7 +6210,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>3496</v>
+        <v>3573</v>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
@@ -6218,7 +6218,7 @@
 IDENTITY: a fierce woman in her late thirties of Brazilian Amazonian heritage with long braided hair.
 BODY: tall and lean with wide shoulders, long ropy arms, a huge feathered cloak build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. agile mover.
 FACE: fierce, delighted.
-COSTUME: tall woman with an antler crown and braided hair in a green leaf-cloak and straps, a carved horn at her lips, a fox, an owl, a small panther and a monkey gathered at her feet and shoulders. Signature exaggeration: an enormous feathered cloak, a huge carved horn at the lips and a tall antler crown.
+COSTUME: tall woman with an antler crown and long black braids, a huge maroon-and-gold feather cloak with green leaf trim, a claw-tooth belt and striped boots, a big carved horn at her lips, an owl on her shoulder, a monkey on her back, a black panther and a fox at her feet. Signature exaggeration: an enormous feathered cloak, a huge carved horn at the lips and a tall antler crown.
 POSE: striding forward blowing the horn, the animals fanned out around her. Pose energy: arms flung wide or one hand commanding, small summoned allies bursting out around the figure drawn small and clearly separate, a strong S-curve body. Head turned toward the viewer. The pose must say "summoner" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -6240,7 +6240,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a drowned suburb overtaken by forest: roots through a server room, mossy satellite dishes, ferns on car roofs, low mist.
-Scene props for Canopy Beastmasters: a rope-bridge canopy village with a giant tree trunk, hanging fruit lamps, vine ladders and a wide leafy clearing. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Canopy Beastmasters: a rope-bridge canopy village around a giant tree trunk under a pale moon, thatched treehouses with glowing windows, hanging fruit lamps, maroon banners with a tree sigil, waterfalls, clay pots and a wide wooden clearing. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a MOSS-WASHED scene. The people color #3f7d45 washes the whole scene (deep MOSS GREEN: green-tinted sky and mist, mossy green light and shadows on everything), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #6f2a31 for the largest sign, banner or lit window band, SECONDARY #f2c14e for several medium panels, flags or lights, POP #23b04a for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Sticky Wizards: new Shard Cel portrait and background; art text matched
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -4783,7 +4783,7 @@
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>lanky bareheaded human wizard in a patched laboratory robe, messy hair, a bandolier of goo jars across the chest, a sling-staff aimed mid-shot and a confident grin; at his feet a small round green frog wearing a floppy oversized pointed wizard hat, looking up proudly</t>
+          <t>lanky bareheaded human wizard in a patched laboratory robe, messy brown hair and a beard, a green-and-gold robe, a bandolier of goo jars across the chest, a sling-staff aimed mid-shot and a confident grin; at his feet a small round green frog wearing a floppy oversized pointed wizard hat, looking up proudly</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -6674,7 +6674,7 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>3737</v>
+        <v>3778</v>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
@@ -6682,7 +6682,7 @@
 IDENTITY: Sticky Wizard (created by Mike Mears): a lanky, hatless male wizard in his thirties with messy hair and a playful, capable manner, and at his feet a small round frog wearing the wizard hat.
 BODY: tall and lanky build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. agile mover.
 FACE: cheerful, wide-eyed confidence; the frog looks smug under the hat.
-COSTUME: lanky bareheaded human wizard in a patched laboratory robe, messy hair, a bandolier of goo jars across the chest, a sling-staff aimed mid-shot and a confident grin; at his feet a small round green frog wearing a floppy oversized pointed wizard hat, looking up proudly. Signature exaggeration: a giant goo sling-staff aimed toward the viewer, an oversized bandolier of goo jars and a huge floppy frog hat.
+COSTUME: lanky bareheaded human wizard in a patched laboratory robe, messy brown hair and a beard, a green-and-gold robe, a bandolier of goo jars across the chest, a sling-staff aimed mid-shot and a confident grin; at his feet a small round green frog wearing a floppy oversized pointed wizard hat, looking up proudly. Signature exaggeration: a giant goo sling-staff aimed toward the viewer, an oversized bandolier of goo jars and a huge floppy frog hat.
 POSE: leaning into a sling-shot of goo, the hatless wizard mid-stride while the frog at his feet holds its hat on with one hand. Pose energy: a braced aggressive firing or throwing stance, the weapon or throwing arm foreshortened toward the viewer, back arched, the muzzle or throw clearly readable. Head turned toward the viewer. The pose must say "blaster" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
@@ -6704,7 +6704,7 @@
         <is>
           <t>Bold flat-shape 2D illustration, 16:9 landscape. Layered flat color shapes in three depth planes: near black silhouette shapes at the edges, mid shapes in the people color, far shapes in a pale haze of the same color. Sharp angular architecture built from wedges and slabs with hard-edged black shadow shapes. The sky is two or three flat color bands with one flat moon disc. Thin flat rim-light shapes on edges and flat glow discs behind lamps. No stippling, no grain, no smudge, no halftone, no gradients, no blur.
 Setting: a ruined broadcast-and-ritual precinct: a leaning radio-tower observatory, a mushroom-furred factory floor, a chalk summoning circle on cracked concrete, a broken substation, drifting arcane glow.
-Scene props for Sticky Wizards: a flooded alchemy basement with bubbling goo vats, dripping pipes, glued-down furniture and shelves of jars. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
+Scene props for Sticky Wizards: a flooded alchemy lab under a violet moon with tall glowing green goo vats, dripping pipes, a shelf of colorful jars, glowing pink mushrooms, a leaning radio-tower spire, waterfalls and lanterns. These are things the character could never wear or carry, so they live in the environment as set dressing on the left, right and far plane, tied to the setting, with nobody using them.
 Keep the center-lower area open for the character. Props on the left, right and far plane only. Horizon at one-third height, a flat moon disc upper-left, ruined shapes receding to the left.
 COLOR (most important): a VIOLET-WASHED scene. The people color #6b3fa6 washes the whole scene (rich VIOLET: purple sky, violet haze, violet-tinted light and shadows on everything), about 65% of the image, as flat bands and shapes in light-to-dark steps across sky, haze, ground and walls. 
 TRIO ACCENTS (clearly visible, about 20% of the image combined, never tiny): MAIN #0de609 for the largest sign, banner or lit window band, SECONDARY #ffd23f for several medium panels, flags or lights, POP #ff6b9d for a handful of small bright sparks. Place at least two accents on the foreground props and reflect them on the ground as flat shapes. Do not let the accents vanish and do not make the scene mostly grey.

</xml_diff>

<commit_message>
Pinball Gunners: new Shard Cel portrait; description and pose matched to the art
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NDA_MVP_Characters_V2.xlsx
+++ b/NDA_MVP_Characters_V2.xlsx
@@ -1648,7 +1648,7 @@
       </c>
       <c r="Q3" s="6" t="inlineStr">
         <is>
-          <t>rangy young woman with a high dark dreadlock bun and a blue bandana, a hot-pink cape-jacket with blue lightning trim, a star-emblem round bumper shield on one arm, a long pink-and-cream railgun rifle with plunger-tipped barrel and scope aimed in both hands, a plunger-tipped spear slung across the back, studded belt, star knee-guard and laced boots</t>
+          <t>rangy young woman with a high dark dreadlock bun and a blue bandana, a hot-pink cape-jacket with blue lightning trim, a round cream-and-cyan arcade-chip bumper shield raised on one arm, a long pink-and-cream railgun rifle with a hexagonal glowing muzzle and a scope, aimed one-handed, a plunger-tipped spear slung across the back, studded belt, geometric knee-guard and laced boots</t>
         </is>
       </c>
       <c r="R3" s="6" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
-          <t>braced low on one knee, the railgun shouldered and angled for a bank shot, the bumper shield raised on the other arm</t>
+          <t>wide lunge on planted boots, the railgun levelled at the viewer for a bank shot, the bumper shield raised on the other arm</t>
         </is>
       </c>
       <c r="T3" s="6" t="inlineStr">
@@ -5204,15 +5204,15 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>3598</v>
+        <v>3636</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Pinball Gunners: a blaster (ranged firepower and explosive area damage), combat character, Human › Arcade Clans.
 BODY: rangy and loose-limbed build. Proportion recipe: medium heroic build: head one sixth of the height, long limbs, big hands and feet. agile mover.
 FACE: gleeful squint, one eye closed to aim.
-COSTUME: rangy young woman with a high dark dreadlock bun and a blue bandana, a hot-pink cape-jacket with blue lightning trim, a star-emblem round bumper shield on one arm, a long pink-and-cream railgun rifle with plunger-tipped barrel and scope aimed in both hands, a plunger-tipped spear slung across the back, studded belt, star knee-guard and laced boots. Signature exaggeration: an enormous gloved trigger hand and the plunger-tipped rifle muzzle pushed toward the viewer, giant sneakers.
-POSE: braced low on one knee, the railgun shouldered and angled for a bank shot, the bumper shield raised on the other arm. Pose energy: a braced aggressive firing or throwing stance, the weapon or throwing arm foreshortened toward the viewer, back arched, the muzzle or throw clearly readable. Head turned toward the viewer. The pose must say "blaster" at a glance.
+COSTUME: rangy young woman with a high dark dreadlock bun and a blue bandana, a hot-pink cape-jacket with blue lightning trim, a round cream-and-cyan arcade-chip bumper shield raised on one arm, a long pink-and-cream railgun rifle with a hexagonal glowing muzzle and a scope, aimed one-handed, a plunger-tipped spear slung across the back, studded belt, geometric knee-guard and laced boots. Signature exaggeration: an enormous gloved trigger hand and the plunger-tipped rifle muzzle pushed toward the viewer, giant sneakers.
+POSE: wide lunge on planted boots, the railgun levelled at the viewer for a bank shot, the bumper shield raised on the other arm. Pose energy: a braced aggressive firing or throwing stance, the weapon or throwing arm foreshortened toward the viewer, back arched, the muzzle or throw clearly readable. Head turned toward the viewer. The pose must say "blaster" at a glance.
 STYLE KIT (Shard Cel 2.0):
 Shape language: sharp angular shards, wedges and triangles. Hair, cloth hems, capes and tails end in long pointed blades. The silhouette reads instantly, even as a tiny thumbnail.
 Stylized heroic proportions: small head, broad shoulders, tapered waist, long elastic limbs, and hands and feet oversized to about one and a half times natural size.

</xml_diff>